<commit_message>
Update historical price analysis 2026-03
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Monthly Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Heatmap" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: rebuild all outputs from freshly downloaded raw data
Forced re-download of every AEMO file (1,372 region-months, 0 errors). Every price, count and
flag is identical to the previous outputs on all 1,372 common rows, so AEMO has revised nothing
and the CPI parser change moves no real price. The only row change: TAS 2005-05 (partial month)
is no longer published. Workbooks gain the n/a rolling rows, the CPI Estimated column and the
real-dollar note.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -616,10 +616,55 @@
         <v>134.45</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>15-Year Average</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>80.61</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>93.34</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>98.20999999999999</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>113.53</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>20-Year Average</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>71.44</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>85.43000000000001</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>91.25</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>109.84</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Data through: Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Real prices are in Jun 2026 dollars (latest published CPI quarter). The latest 3 month(s) have no CPI yet, so real = nominal there (flagged in Monthly Data).</t>
         </is>
       </c>
     </row>
@@ -634,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F280"/>
+  <dimension ref="A1:G280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -643,6 +688,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -676,6 +722,11 @@
           <t>Carbon Tax</t>
         </is>
       </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>CPI Estimated</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -696,6 +747,7 @@
         <v>141.85</v>
       </c>
       <c r="F2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -716,6 +768,7 @@
         <v>41.13</v>
       </c>
       <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -736,6 +789,7 @@
         <v>48.89</v>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -756,6 +810,7 @@
         <v>36.01</v>
       </c>
       <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -776,6 +831,7 @@
         <v>38.33</v>
       </c>
       <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -796,6 +852,7 @@
         <v>54.88</v>
       </c>
       <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -816,6 +873,7 @@
         <v>58.1</v>
       </c>
       <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -836,6 +894,7 @@
         <v>89.73999999999999</v>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -856,6 +915,7 @@
         <v>213.84</v>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -876,6 +936,7 @@
         <v>68.45</v>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -896,6 +957,7 @@
         <v>68.98</v>
       </c>
       <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -916,6 +978,7 @@
         <v>61.55</v>
       </c>
       <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -936,6 +999,7 @@
         <v>79.59</v>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -956,6 +1020,7 @@
         <v>47.62</v>
       </c>
       <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -976,6 +1041,7 @@
         <v>58.33</v>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -996,6 +1062,7 @@
         <v>227.63</v>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1016,6 +1083,7 @@
         <v>237.09</v>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1036,6 +1104,7 @@
         <v>199.89</v>
       </c>
       <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1056,6 +1125,7 @@
         <v>118.22</v>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
+      <c r="G20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1076,6 +1146,7 @@
         <v>90.86</v>
       </c>
       <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1096,6 +1167,7 @@
         <v>35.5</v>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1116,6 +1188,7 @@
         <v>65.18000000000001</v>
       </c>
       <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1136,6 +1209,7 @@
         <v>49.19</v>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1156,6 +1230,7 @@
         <v>57.62</v>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
+      <c r="G25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1176,6 +1251,7 @@
         <v>49.13</v>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
+      <c r="G26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1196,6 +1272,7 @@
         <v>65.25</v>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
+      <c r="G27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1216,6 +1293,7 @@
         <v>63.66</v>
       </c>
       <c r="F28" s="7" t="inlineStr"/>
+      <c r="G28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1236,6 +1314,7 @@
         <v>151.86</v>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
+      <c r="G29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1256,6 +1335,7 @@
         <v>182.76</v>
       </c>
       <c r="F30" s="7" t="inlineStr"/>
+      <c r="G30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1276,6 +1356,7 @@
         <v>224.06</v>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
+      <c r="G31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1296,6 +1377,7 @@
         <v>59.26</v>
       </c>
       <c r="F32" s="7" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1316,6 +1398,7 @@
         <v>214.04</v>
       </c>
       <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1336,6 +1419,7 @@
         <v>47.48</v>
       </c>
       <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1356,6 +1440,7 @@
         <v>40.96</v>
       </c>
       <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1376,6 +1461,7 @@
         <v>55.47</v>
       </c>
       <c r="F36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1396,6 +1482,7 @@
         <v>65.97</v>
       </c>
       <c r="F37" s="7" t="inlineStr"/>
+      <c r="G37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1416,6 +1503,7 @@
         <v>125.74</v>
       </c>
       <c r="F38" s="7" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1436,6 +1524,7 @@
         <v>60.07</v>
       </c>
       <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1456,6 +1545,7 @@
         <v>58.6</v>
       </c>
       <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -1476,6 +1566,7 @@
         <v>52.42</v>
       </c>
       <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1496,6 +1587,7 @@
         <v>68.89</v>
       </c>
       <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1516,6 +1608,7 @@
         <v>42.67</v>
       </c>
       <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -1536,6 +1629,7 @@
         <v>151.88</v>
       </c>
       <c r="F44" s="7" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -1556,6 +1650,7 @@
         <v>106.17</v>
       </c>
       <c r="F45" s="7" t="inlineStr"/>
+      <c r="G45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -1576,6 +1671,7 @@
         <v>106.58</v>
       </c>
       <c r="F46" s="7" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -1596,6 +1692,7 @@
         <v>171.89</v>
       </c>
       <c r="F47" s="7" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1616,6 +1713,7 @@
         <v>126.78</v>
       </c>
       <c r="F48" s="7" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -1636,6 +1734,7 @@
         <v>667.89</v>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
+      <c r="G49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -1656,6 +1755,7 @@
         <v>176.55</v>
       </c>
       <c r="F50" s="7" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -1676,6 +1776,7 @@
         <v>78.26000000000001</v>
       </c>
       <c r="F51" s="7" t="inlineStr"/>
+      <c r="G51" s="7" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -1696,6 +1797,7 @@
         <v>100.04</v>
       </c>
       <c r="F52" s="7" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -1716,6 +1818,7 @@
         <v>92.3</v>
       </c>
       <c r="F53" s="7" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -1736,6 +1839,7 @@
         <v>78.84999999999999</v>
       </c>
       <c r="F54" s="7" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -1756,6 +1860,7 @@
         <v>91.28</v>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -1776,6 +1881,7 @@
         <v>71.67</v>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -1796,6 +1902,7 @@
         <v>52.12</v>
       </c>
       <c r="F57" s="7" t="inlineStr"/>
+      <c r="G57" s="7" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -1816,6 +1923,7 @@
         <v>76.63</v>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -1836,6 +1944,7 @@
         <v>64.55</v>
       </c>
       <c r="F59" s="7" t="inlineStr"/>
+      <c r="G59" s="7" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -1856,6 +1965,7 @@
         <v>84.69</v>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
+      <c r="G60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -1876,6 +1986,7 @@
         <v>81.91</v>
       </c>
       <c r="F61" s="7" t="inlineStr"/>
+      <c r="G61" s="7" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -1896,6 +2007,7 @@
         <v>88.59</v>
       </c>
       <c r="F62" s="7" t="inlineStr"/>
+      <c r="G62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -1916,6 +2028,7 @@
         <v>77.11</v>
       </c>
       <c r="F63" s="7" t="inlineStr"/>
+      <c r="G63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -1936,6 +2049,7 @@
         <v>72.08</v>
       </c>
       <c r="F64" s="7" t="inlineStr"/>
+      <c r="G64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -1956,6 +2070,7 @@
         <v>226.53</v>
       </c>
       <c r="F65" s="7" t="inlineStr"/>
+      <c r="G65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -1976,6 +2091,7 @@
         <v>60.43</v>
       </c>
       <c r="F66" s="7" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -1996,6 +2112,7 @@
         <v>44.2</v>
       </c>
       <c r="F67" s="7" t="inlineStr"/>
+      <c r="G67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -2016,6 +2133,7 @@
         <v>116.01</v>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
+      <c r="G68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -2036,6 +2154,7 @@
         <v>62.06</v>
       </c>
       <c r="F69" s="7" t="inlineStr"/>
+      <c r="G69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -2056,6 +2175,7 @@
         <v>46.78</v>
       </c>
       <c r="F70" s="7" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -2076,6 +2196,7 @@
         <v>74.93000000000001</v>
       </c>
       <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -2096,6 +2217,7 @@
         <v>56.39</v>
       </c>
       <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -2116,6 +2238,7 @@
         <v>72.48</v>
       </c>
       <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -2136,6 +2259,7 @@
         <v>63.34</v>
       </c>
       <c r="F74" s="7" t="inlineStr"/>
+      <c r="G74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -2156,6 +2280,7 @@
         <v>43.41</v>
       </c>
       <c r="F75" s="7" t="inlineStr"/>
+      <c r="G75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -2176,6 +2301,7 @@
         <v>44.75</v>
       </c>
       <c r="F76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -2196,6 +2322,7 @@
         <v>50.09</v>
       </c>
       <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="7" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -2216,6 +2343,7 @@
         <v>327.39</v>
       </c>
       <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -2236,6 +2364,7 @@
         <v>290.91</v>
       </c>
       <c r="F79" s="7" t="inlineStr"/>
+      <c r="G79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -2256,6 +2385,7 @@
         <v>122.31</v>
       </c>
       <c r="F80" s="7" t="inlineStr"/>
+      <c r="G80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -2276,6 +2406,7 @@
         <v>149.86</v>
       </c>
       <c r="F81" s="7" t="inlineStr"/>
+      <c r="G81" s="7" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -2296,6 +2427,7 @@
         <v>47.57</v>
       </c>
       <c r="F82" s="7" t="inlineStr"/>
+      <c r="G82" s="7" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -2316,6 +2448,7 @@
         <v>43.76</v>
       </c>
       <c r="F83" s="7" t="inlineStr"/>
+      <c r="G83" s="7" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -2336,6 +2469,7 @@
         <v>47.57</v>
       </c>
       <c r="F84" s="7" t="inlineStr"/>
+      <c r="G84" s="7" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -2356,6 +2490,7 @@
         <v>59.86</v>
       </c>
       <c r="F85" s="7" t="inlineStr"/>
+      <c r="G85" s="7" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -2376,6 +2511,7 @@
         <v>45.06</v>
       </c>
       <c r="F86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -2396,6 +2532,7 @@
         <v>71.38</v>
       </c>
       <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -2416,6 +2553,7 @@
         <v>39.21</v>
       </c>
       <c r="F88" s="7" t="inlineStr"/>
+      <c r="G88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -2436,6 +2574,7 @@
         <v>36.66</v>
       </c>
       <c r="F89" s="7" t="inlineStr"/>
+      <c r="G89" s="7" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -2456,6 +2595,7 @@
         <v>36.81</v>
       </c>
       <c r="F90" s="7" t="inlineStr"/>
+      <c r="G90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -2476,6 +2616,7 @@
         <v>37.72</v>
       </c>
       <c r="F91" s="7" t="inlineStr"/>
+      <c r="G91" s="7" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -2496,6 +2637,7 @@
         <v>117.81</v>
       </c>
       <c r="F92" s="7" t="inlineStr"/>
+      <c r="G92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -2516,6 +2658,7 @@
         <v>389.69</v>
       </c>
       <c r="F93" s="7" t="inlineStr"/>
+      <c r="G93" s="7" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -2536,6 +2679,7 @@
         <v>43.55</v>
       </c>
       <c r="F94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -2556,6 +2700,7 @@
         <v>40.63</v>
       </c>
       <c r="F95" s="7" t="inlineStr"/>
+      <c r="G95" s="7" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -2576,6 +2721,7 @@
         <v>45.02</v>
       </c>
       <c r="F96" s="7" t="inlineStr"/>
+      <c r="G96" s="7" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -2596,6 +2742,7 @@
         <v>44.07</v>
       </c>
       <c r="F97" s="7" t="inlineStr"/>
+      <c r="G97" s="7" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -2616,6 +2763,7 @@
         <v>51.8</v>
       </c>
       <c r="F98" s="7" t="inlineStr"/>
+      <c r="G98" s="7" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -2636,6 +2784,7 @@
         <v>48.51</v>
       </c>
       <c r="F99" s="7" t="inlineStr"/>
+      <c r="G99" s="7" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -2656,6 +2805,7 @@
         <v>45.55</v>
       </c>
       <c r="F100" s="7" t="inlineStr"/>
+      <c r="G100" s="7" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -2676,6 +2826,7 @@
         <v>44.63</v>
       </c>
       <c r="F101" s="7" t="inlineStr"/>
+      <c r="G101" s="7" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -2696,6 +2847,7 @@
         <v>69.92</v>
       </c>
       <c r="F102" s="7" t="inlineStr"/>
+      <c r="G102" s="7" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -2716,6 +2868,7 @@
         <v>40.37</v>
       </c>
       <c r="F103" s="7" t="inlineStr"/>
+      <c r="G103" s="7" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -2736,6 +2889,7 @@
         <v>41.73</v>
       </c>
       <c r="F104" s="7" t="inlineStr"/>
+      <c r="G104" s="7" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -2756,6 +2910,7 @@
         <v>43.17</v>
       </c>
       <c r="F105" s="7" t="inlineStr"/>
+      <c r="G105" s="7" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -2776,6 +2931,7 @@
         <v>41.16</v>
       </c>
       <c r="F106" s="7" t="inlineStr"/>
+      <c r="G106" s="7" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -2796,6 +2952,7 @@
         <v>53.95</v>
       </c>
       <c r="F107" s="7" t="inlineStr"/>
+      <c r="G107" s="7" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -2816,6 +2973,7 @@
         <v>44.82</v>
       </c>
       <c r="F108" s="7" t="inlineStr"/>
+      <c r="G108" s="7" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -2836,6 +2994,7 @@
         <v>59.33</v>
       </c>
       <c r="F109" s="7" t="inlineStr"/>
+      <c r="G109" s="7" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
@@ -2860,6 +3019,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G110" s="10" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
@@ -2884,6 +3044,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G111" s="10" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
@@ -2908,6 +3069,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G112" s="10" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
@@ -2932,6 +3094,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G113" s="10" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
@@ -2956,6 +3119,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G114" s="10" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
@@ -2980,6 +3144,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G115" s="10" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
@@ -3004,6 +3169,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G116" s="10" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
@@ -3028,6 +3194,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G117" s="10" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
@@ -3052,6 +3219,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
@@ -3076,6 +3244,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G119" s="10" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
@@ -3100,6 +3269,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G120" s="10" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
@@ -3124,6 +3294,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G121" s="10" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
@@ -3148,6 +3319,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G122" s="10" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
@@ -3172,6 +3344,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G123" s="10" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
@@ -3196,6 +3369,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G124" s="10" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
@@ -3220,6 +3394,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G125" s="10" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
@@ -3244,6 +3419,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G126" s="10" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
@@ -3268,6 +3444,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G127" s="10" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
@@ -3292,6 +3469,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G128" s="10" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
@@ -3316,6 +3494,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
@@ -3340,6 +3519,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
@@ -3364,6 +3544,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
@@ -3388,6 +3569,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
@@ -3412,6 +3594,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -3432,6 +3615,7 @@
         <v>61.6</v>
       </c>
       <c r="F134" s="7" t="inlineStr"/>
+      <c r="G134" s="7" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -3452,6 +3636,7 @@
         <v>55.17</v>
       </c>
       <c r="F135" s="7" t="inlineStr"/>
+      <c r="G135" s="7" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -3472,6 +3657,7 @@
         <v>61.15</v>
       </c>
       <c r="F136" s="7" t="inlineStr"/>
+      <c r="G136" s="7" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -3492,6 +3678,7 @@
         <v>46.89</v>
       </c>
       <c r="F137" s="7" t="inlineStr"/>
+      <c r="G137" s="7" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -3512,6 +3699,7 @@
         <v>56.35</v>
       </c>
       <c r="F138" s="7" t="inlineStr"/>
+      <c r="G138" s="7" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -3532,6 +3720,7 @@
         <v>48.34</v>
       </c>
       <c r="F139" s="7" t="inlineStr"/>
+      <c r="G139" s="7" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -3552,6 +3741,7 @@
         <v>64.94</v>
       </c>
       <c r="F140" s="7" t="inlineStr"/>
+      <c r="G140" s="7" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -3572,6 +3762,7 @@
         <v>53.16</v>
       </c>
       <c r="F141" s="7" t="inlineStr"/>
+      <c r="G141" s="7" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -3592,6 +3783,7 @@
         <v>48</v>
       </c>
       <c r="F142" s="7" t="inlineStr"/>
+      <c r="G142" s="7" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -3612,6 +3804,7 @@
         <v>58.11</v>
       </c>
       <c r="F143" s="7" t="inlineStr"/>
+      <c r="G143" s="7" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -3632,6 +3825,7 @@
         <v>56.24</v>
       </c>
       <c r="F144" s="7" t="inlineStr"/>
+      <c r="G144" s="7" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -3652,6 +3846,7 @@
         <v>54.92</v>
       </c>
       <c r="F145" s="7" t="inlineStr"/>
+      <c r="G145" s="7" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -3672,6 +3867,7 @@
         <v>59.25</v>
       </c>
       <c r="F146" s="7" t="inlineStr"/>
+      <c r="G146" s="7" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -3692,6 +3888,7 @@
         <v>54.54</v>
       </c>
       <c r="F147" s="7" t="inlineStr"/>
+      <c r="G147" s="7" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -3712,6 +3909,7 @@
         <v>104.59</v>
       </c>
       <c r="F148" s="7" t="inlineStr"/>
+      <c r="G148" s="7" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -3732,6 +3930,7 @@
         <v>56.65</v>
       </c>
       <c r="F149" s="7" t="inlineStr"/>
+      <c r="G149" s="7" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -3752,6 +3951,7 @@
         <v>83.95</v>
       </c>
       <c r="F150" s="7" t="inlineStr"/>
+      <c r="G150" s="7" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -3772,6 +3972,7 @@
         <v>68.48</v>
       </c>
       <c r="F151" s="7" t="inlineStr"/>
+      <c r="G151" s="7" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -3792,6 +3993,7 @@
         <v>82.09999999999999</v>
       </c>
       <c r="F152" s="7" t="inlineStr"/>
+      <c r="G152" s="7" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -3812,6 +4014,7 @@
         <v>61.97</v>
       </c>
       <c r="F153" s="7" t="inlineStr"/>
+      <c r="G153" s="7" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -3832,6 +4035,7 @@
         <v>66.41</v>
       </c>
       <c r="F154" s="7" t="inlineStr"/>
+      <c r="G154" s="7" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -3852,6 +4056,7 @@
         <v>100.28</v>
       </c>
       <c r="F155" s="7" t="inlineStr"/>
+      <c r="G155" s="7" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -3872,6 +4077,7 @@
         <v>105.84</v>
       </c>
       <c r="F156" s="7" t="inlineStr"/>
+      <c r="G156" s="7" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -3892,6 +4098,7 @@
         <v>158.99</v>
       </c>
       <c r="F157" s="7" t="inlineStr"/>
+      <c r="G157" s="7" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -3912,6 +4119,7 @@
         <v>113.29</v>
       </c>
       <c r="F158" s="7" t="inlineStr"/>
+      <c r="G158" s="7" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -3932,6 +4140,7 @@
         <v>75.93000000000001</v>
       </c>
       <c r="F159" s="7" t="inlineStr"/>
+      <c r="G159" s="7" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -3952,6 +4161,7 @@
         <v>66.28</v>
       </c>
       <c r="F160" s="7" t="inlineStr"/>
+      <c r="G160" s="7" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -3972,6 +4182,7 @@
         <v>77.73</v>
       </c>
       <c r="F161" s="7" t="inlineStr"/>
+      <c r="G161" s="7" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -3992,6 +4203,7 @@
         <v>151.91</v>
       </c>
       <c r="F162" s="7" t="inlineStr"/>
+      <c r="G162" s="7" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -4012,6 +4224,7 @@
         <v>78.84</v>
       </c>
       <c r="F163" s="7" t="inlineStr"/>
+      <c r="G163" s="7" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -4032,6 +4245,7 @@
         <v>140.81</v>
       </c>
       <c r="F164" s="7" t="inlineStr"/>
+      <c r="G164" s="7" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -4052,6 +4266,7 @@
         <v>370.26</v>
       </c>
       <c r="F165" s="7" t="inlineStr"/>
+      <c r="G165" s="7" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -4072,6 +4287,7 @@
         <v>144.15</v>
       </c>
       <c r="F166" s="7" t="inlineStr"/>
+      <c r="G166" s="7" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -4092,6 +4308,7 @@
         <v>151.65</v>
       </c>
       <c r="F167" s="7" t="inlineStr"/>
+      <c r="G167" s="7" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -4112,6 +4329,7 @@
         <v>126.08</v>
       </c>
       <c r="F168" s="7" t="inlineStr"/>
+      <c r="G168" s="7" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -4132,6 +4350,7 @@
         <v>117.53</v>
       </c>
       <c r="F169" s="7" t="inlineStr"/>
+      <c r="G169" s="7" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -4152,6 +4371,7 @@
         <v>133.84</v>
       </c>
       <c r="F170" s="7" t="inlineStr"/>
+      <c r="G170" s="7" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -4172,6 +4392,7 @@
         <v>144.47</v>
       </c>
       <c r="F171" s="7" t="inlineStr"/>
+      <c r="G171" s="7" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -4192,6 +4413,7 @@
         <v>120.59</v>
       </c>
       <c r="F172" s="7" t="inlineStr"/>
+      <c r="G172" s="7" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -4212,6 +4434,7 @@
         <v>117.88</v>
       </c>
       <c r="F173" s="7" t="inlineStr"/>
+      <c r="G173" s="7" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -4232,6 +4455,7 @@
         <v>114.03</v>
       </c>
       <c r="F174" s="7" t="inlineStr"/>
+      <c r="G174" s="7" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -4252,6 +4476,7 @@
         <v>114.57</v>
       </c>
       <c r="F175" s="7" t="inlineStr"/>
+      <c r="G175" s="7" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -4272,6 +4497,7 @@
         <v>109.52</v>
       </c>
       <c r="F176" s="7" t="inlineStr"/>
+      <c r="G176" s="7" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -4292,6 +4518,7 @@
         <v>104.61</v>
       </c>
       <c r="F177" s="7" t="inlineStr"/>
+      <c r="G177" s="7" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -4312,6 +4539,7 @@
         <v>90.81</v>
       </c>
       <c r="F178" s="7" t="inlineStr"/>
+      <c r="G178" s="7" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -4332,6 +4560,7 @@
         <v>110.71</v>
       </c>
       <c r="F179" s="7" t="inlineStr"/>
+      <c r="G179" s="7" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -4352,6 +4581,7 @@
         <v>112.32</v>
       </c>
       <c r="F180" s="7" t="inlineStr"/>
+      <c r="G180" s="7" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -4372,6 +4602,7 @@
         <v>167.26</v>
       </c>
       <c r="F181" s="7" t="inlineStr"/>
+      <c r="G181" s="7" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -4392,6 +4623,7 @@
         <v>108.36</v>
       </c>
       <c r="F182" s="7" t="inlineStr"/>
+      <c r="G182" s="7" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -4412,6 +4644,7 @@
         <v>137.59</v>
       </c>
       <c r="F183" s="7" t="inlineStr"/>
+      <c r="G183" s="7" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -4432,6 +4665,7 @@
         <v>138.38</v>
       </c>
       <c r="F184" s="7" t="inlineStr"/>
+      <c r="G184" s="7" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -4452,6 +4686,7 @@
         <v>130.23</v>
       </c>
       <c r="F185" s="7" t="inlineStr"/>
+      <c r="G185" s="7" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -4472,6 +4707,7 @@
         <v>127.99</v>
       </c>
       <c r="F186" s="7" t="inlineStr"/>
+      <c r="G186" s="7" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -4492,6 +4728,7 @@
         <v>125.9</v>
       </c>
       <c r="F187" s="7" t="inlineStr"/>
+      <c r="G187" s="7" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -4512,6 +4749,7 @@
         <v>201.99</v>
       </c>
       <c r="F188" s="7" t="inlineStr"/>
+      <c r="G188" s="7" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -4532,6 +4770,7 @@
         <v>131.59</v>
       </c>
       <c r="F189" s="7" t="inlineStr"/>
+      <c r="G189" s="7" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -4552,6 +4791,7 @@
         <v>126.84</v>
       </c>
       <c r="F190" s="7" t="inlineStr"/>
+      <c r="G190" s="7" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -4572,6 +4812,7 @@
         <v>112.17</v>
       </c>
       <c r="F191" s="7" t="inlineStr"/>
+      <c r="G191" s="7" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -4592,6 +4833,7 @@
         <v>115.59</v>
       </c>
       <c r="F192" s="7" t="inlineStr"/>
+      <c r="G192" s="7" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -4612,6 +4854,7 @@
         <v>135.94</v>
       </c>
       <c r="F193" s="7" t="inlineStr"/>
+      <c r="G193" s="7" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -4632,6 +4875,7 @@
         <v>101.95</v>
       </c>
       <c r="F194" s="7" t="inlineStr"/>
+      <c r="G194" s="7" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -4652,6 +4896,7 @@
         <v>123.27</v>
       </c>
       <c r="F195" s="7" t="inlineStr"/>
+      <c r="G195" s="7" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -4672,6 +4917,7 @@
         <v>137.46</v>
       </c>
       <c r="F196" s="7" t="inlineStr"/>
+      <c r="G196" s="7" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -4692,6 +4938,7 @@
         <v>139.53</v>
       </c>
       <c r="F197" s="7" t="inlineStr"/>
+      <c r="G197" s="7" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -4712,6 +4959,7 @@
         <v>91.01000000000001</v>
       </c>
       <c r="F198" s="7" t="inlineStr"/>
+      <c r="G198" s="7" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -4732,6 +4980,7 @@
         <v>69.3</v>
       </c>
       <c r="F199" s="7" t="inlineStr"/>
+      <c r="G199" s="7" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -4752,6 +5001,7 @@
         <v>234.62</v>
       </c>
       <c r="F200" s="7" t="inlineStr"/>
+      <c r="G200" s="7" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -4772,6 +5022,7 @@
         <v>74.39</v>
       </c>
       <c r="F201" s="7" t="inlineStr"/>
+      <c r="G201" s="7" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
@@ -4792,6 +5043,7 @@
         <v>64.18000000000001</v>
       </c>
       <c r="F202" s="7" t="inlineStr"/>
+      <c r="G202" s="7" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
@@ -4812,6 +5064,7 @@
         <v>57.4</v>
       </c>
       <c r="F203" s="7" t="inlineStr"/>
+      <c r="G203" s="7" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
@@ -4832,6 +5085,7 @@
         <v>61.49</v>
       </c>
       <c r="F204" s="7" t="inlineStr"/>
+      <c r="G204" s="7" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -4852,6 +5106,7 @@
         <v>76.98</v>
       </c>
       <c r="F205" s="7" t="inlineStr"/>
+      <c r="G205" s="7" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
@@ -4872,6 +5127,7 @@
         <v>71.11</v>
       </c>
       <c r="F206" s="7" t="inlineStr"/>
+      <c r="G206" s="7" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -4892,6 +5148,7 @@
         <v>75.41</v>
       </c>
       <c r="F207" s="7" t="inlineStr"/>
+      <c r="G207" s="7" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
@@ -4912,6 +5169,7 @@
         <v>55.54</v>
       </c>
       <c r="F208" s="7" t="inlineStr"/>
+      <c r="G208" s="7" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
@@ -4932,6 +5190,7 @@
         <v>88.5</v>
       </c>
       <c r="F209" s="7" t="inlineStr"/>
+      <c r="G209" s="7" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -4952,6 +5211,7 @@
         <v>103.51</v>
       </c>
       <c r="F210" s="7" t="inlineStr"/>
+      <c r="G210" s="7" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -4972,6 +5232,7 @@
         <v>134.44</v>
       </c>
       <c r="F211" s="7" t="inlineStr"/>
+      <c r="G211" s="7" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -4992,6 +5253,7 @@
         <v>53.84</v>
       </c>
       <c r="F212" s="7" t="inlineStr"/>
+      <c r="G212" s="7" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
@@ -5012,6 +5274,7 @@
         <v>45.1</v>
       </c>
       <c r="F213" s="7" t="inlineStr"/>
+      <c r="G213" s="7" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
@@ -5032,6 +5295,7 @@
         <v>49.46</v>
       </c>
       <c r="F214" s="7" t="inlineStr"/>
+      <c r="G214" s="7" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -5052,6 +5316,7 @@
         <v>82.88</v>
       </c>
       <c r="F215" s="7" t="inlineStr"/>
+      <c r="G215" s="7" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
@@ -5072,6 +5337,7 @@
         <v>225</v>
       </c>
       <c r="F216" s="7" t="inlineStr"/>
+      <c r="G216" s="7" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
@@ -5092,6 +5358,7 @@
         <v>313.99</v>
       </c>
       <c r="F217" s="7" t="inlineStr"/>
+      <c r="G217" s="7" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
@@ -5112,6 +5379,7 @@
         <v>214.11</v>
       </c>
       <c r="F218" s="7" t="inlineStr"/>
+      <c r="G218" s="7" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -5132,6 +5400,7 @@
         <v>80.84999999999999</v>
       </c>
       <c r="F219" s="7" t="inlineStr"/>
+      <c r="G219" s="7" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
@@ -5152,6 +5421,7 @@
         <v>58.23</v>
       </c>
       <c r="F220" s="7" t="inlineStr"/>
+      <c r="G220" s="7" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
@@ -5172,6 +5442,7 @@
         <v>72.39</v>
       </c>
       <c r="F221" s="7" t="inlineStr"/>
+      <c r="G221" s="7" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
@@ -5192,6 +5463,7 @@
         <v>88.41</v>
       </c>
       <c r="F222" s="7" t="inlineStr"/>
+      <c r="G222" s="7" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
@@ -5212,6 +5484,7 @@
         <v>84.09</v>
       </c>
       <c r="F223" s="7" t="inlineStr"/>
+      <c r="G223" s="7" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
@@ -5232,6 +5505,7 @@
         <v>97.97</v>
       </c>
       <c r="F224" s="7" t="inlineStr"/>
+      <c r="G224" s="7" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
@@ -5252,6 +5526,7 @@
         <v>110.58</v>
       </c>
       <c r="F225" s="7" t="inlineStr"/>
+      <c r="G225" s="7" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
@@ -5272,6 +5547,7 @@
         <v>124.28</v>
       </c>
       <c r="F226" s="7" t="inlineStr"/>
+      <c r="G226" s="7" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
@@ -5292,6 +5568,7 @@
         <v>240.92</v>
       </c>
       <c r="F227" s="7" t="inlineStr"/>
+      <c r="G227" s="7" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
@@ -5312,6 +5589,7 @@
         <v>452.4</v>
       </c>
       <c r="F228" s="7" t="inlineStr"/>
+      <c r="G228" s="7" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
@@ -5332,6 +5610,7 @@
         <v>514.29</v>
       </c>
       <c r="F229" s="7" t="inlineStr"/>
+      <c r="G229" s="7" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
@@ -5352,6 +5631,7 @@
         <v>493.31</v>
       </c>
       <c r="F230" s="7" t="inlineStr"/>
+      <c r="G230" s="7" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
@@ -5372,6 +5652,7 @@
         <v>180.03</v>
       </c>
       <c r="F231" s="7" t="inlineStr"/>
+      <c r="G231" s="7" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
@@ -5392,6 +5673,7 @@
         <v>180.21</v>
       </c>
       <c r="F232" s="7" t="inlineStr"/>
+      <c r="G232" s="7" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
@@ -5412,6 +5694,7 @@
         <v>177.71</v>
       </c>
       <c r="F233" s="7" t="inlineStr"/>
+      <c r="G233" s="7" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
@@ -5432,6 +5715,7 @@
         <v>121.31</v>
       </c>
       <c r="F234" s="7" t="inlineStr"/>
+      <c r="G234" s="7" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
@@ -5452,6 +5736,7 @@
         <v>82.23</v>
       </c>
       <c r="F235" s="7" t="inlineStr"/>
+      <c r="G235" s="7" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
@@ -5472,6 +5757,7 @@
         <v>107.75</v>
       </c>
       <c r="F236" s="7" t="inlineStr"/>
+      <c r="G236" s="7" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
@@ -5492,6 +5778,7 @@
         <v>107.49</v>
       </c>
       <c r="F237" s="7" t="inlineStr"/>
+      <c r="G237" s="7" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
@@ -5512,6 +5799,7 @@
         <v>149.83</v>
       </c>
       <c r="F238" s="7" t="inlineStr"/>
+      <c r="G238" s="7" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
@@ -5532,6 +5820,7 @@
         <v>128.94</v>
       </c>
       <c r="F239" s="7" t="inlineStr"/>
+      <c r="G239" s="7" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
@@ -5552,6 +5841,7 @@
         <v>253.8</v>
       </c>
       <c r="F240" s="7" t="inlineStr"/>
+      <c r="G240" s="7" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
@@ -5572,6 +5862,7 @@
         <v>136.04</v>
       </c>
       <c r="F241" s="7" t="inlineStr"/>
+      <c r="G241" s="7" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
@@ -5592,6 +5883,7 @@
         <v>102.35</v>
       </c>
       <c r="F242" s="7" t="inlineStr"/>
+      <c r="G242" s="7" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
@@ -5612,6 +5904,7 @@
         <v>113.84</v>
       </c>
       <c r="F243" s="7" t="inlineStr"/>
+      <c r="G243" s="7" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
@@ -5632,6 +5925,7 @@
         <v>76.59</v>
       </c>
       <c r="F244" s="7" t="inlineStr"/>
+      <c r="G244" s="7" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
@@ -5652,6 +5946,7 @@
         <v>45.7</v>
       </c>
       <c r="F245" s="7" t="inlineStr"/>
+      <c r="G245" s="7" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
@@ -5672,6 +5967,7 @@
         <v>102.51</v>
       </c>
       <c r="F246" s="7" t="inlineStr"/>
+      <c r="G246" s="7" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
@@ -5692,6 +5988,7 @@
         <v>88.61</v>
       </c>
       <c r="F247" s="7" t="inlineStr"/>
+      <c r="G247" s="7" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
@@ -5712,6 +6009,7 @@
         <v>86.97</v>
       </c>
       <c r="F248" s="7" t="inlineStr"/>
+      <c r="G248" s="7" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
@@ -5732,6 +6030,7 @@
         <v>173.13</v>
       </c>
       <c r="F249" s="7" t="inlineStr"/>
+      <c r="G249" s="7" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
@@ -5752,6 +6051,7 @@
         <v>75.53</v>
       </c>
       <c r="F250" s="7" t="inlineStr"/>
+      <c r="G250" s="7" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
@@ -5772,6 +6072,7 @@
         <v>91.98</v>
       </c>
       <c r="F251" s="7" t="inlineStr"/>
+      <c r="G251" s="7" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
@@ -5792,6 +6093,7 @@
         <v>453.47</v>
       </c>
       <c r="F252" s="7" t="inlineStr"/>
+      <c r="G252" s="7" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
@@ -5812,6 +6114,7 @@
         <v>183.91</v>
       </c>
       <c r="F253" s="7" t="inlineStr"/>
+      <c r="G253" s="7" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
@@ -5832,6 +6135,7 @@
         <v>164.11</v>
       </c>
       <c r="F254" s="7" t="inlineStr"/>
+      <c r="G254" s="7" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
@@ -5852,6 +6156,7 @@
         <v>267.86</v>
       </c>
       <c r="F255" s="7" t="inlineStr"/>
+      <c r="G255" s="7" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
@@ -5872,6 +6177,7 @@
         <v>52.39</v>
       </c>
       <c r="F256" s="7" t="inlineStr"/>
+      <c r="G256" s="7" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
@@ -5892,6 +6198,7 @@
         <v>86.63</v>
       </c>
       <c r="F257" s="7" t="inlineStr"/>
+      <c r="G257" s="7" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
@@ -5912,6 +6219,7 @@
         <v>380.54</v>
       </c>
       <c r="F258" s="7" t="inlineStr"/>
+      <c r="G258" s="7" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
@@ -5932,6 +6240,7 @@
         <v>184.3</v>
       </c>
       <c r="F259" s="7" t="inlineStr"/>
+      <c r="G259" s="7" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
@@ -5952,6 +6261,7 @@
         <v>99.27</v>
       </c>
       <c r="F260" s="7" t="inlineStr"/>
+      <c r="G260" s="7" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
@@ -5972,6 +6282,7 @@
         <v>105.17</v>
       </c>
       <c r="F261" s="7" t="inlineStr"/>
+      <c r="G261" s="7" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
@@ -5992,6 +6303,7 @@
         <v>86.33</v>
       </c>
       <c r="F262" s="7" t="inlineStr"/>
+      <c r="G262" s="7" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
@@ -6012,6 +6324,7 @@
         <v>112.07</v>
       </c>
       <c r="F263" s="7" t="inlineStr"/>
+      <c r="G263" s="7" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
@@ -6032,6 +6345,7 @@
         <v>168.69</v>
       </c>
       <c r="F264" s="7" t="inlineStr"/>
+      <c r="G264" s="7" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
@@ -6052,6 +6366,7 @@
         <v>451.8</v>
       </c>
       <c r="F265" s="7" t="inlineStr"/>
+      <c r="G265" s="7" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
@@ -6072,6 +6387,7 @@
         <v>110.6</v>
       </c>
       <c r="F266" s="7" t="inlineStr"/>
+      <c r="G266" s="7" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
@@ -6092,6 +6408,7 @@
         <v>115.57</v>
       </c>
       <c r="F267" s="7" t="inlineStr"/>
+      <c r="G267" s="7" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
@@ -6112,6 +6429,7 @@
         <v>68.31999999999999</v>
       </c>
       <c r="F268" s="7" t="inlineStr"/>
+      <c r="G268" s="7" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
@@ -6132,6 +6450,7 @@
         <v>77.64</v>
       </c>
       <c r="F269" s="7" t="inlineStr"/>
+      <c r="G269" s="7" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
@@ -6152,6 +6471,7 @@
         <v>85.87</v>
       </c>
       <c r="F270" s="7" t="inlineStr"/>
+      <c r="G270" s="7" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
@@ -6172,6 +6492,7 @@
         <v>79.77</v>
       </c>
       <c r="F271" s="7" t="inlineStr"/>
+      <c r="G271" s="7" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
@@ -6192,6 +6513,7 @@
         <v>46.48</v>
       </c>
       <c r="F272" s="7" t="inlineStr"/>
+      <c r="G272" s="7" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
@@ -6212,6 +6534,7 @@
         <v>98.39</v>
       </c>
       <c r="F273" s="7" t="inlineStr"/>
+      <c r="G273" s="7" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
@@ -6232,6 +6555,7 @@
         <v>71.89</v>
       </c>
       <c r="F274" s="7" t="inlineStr"/>
+      <c r="G274" s="7" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
@@ -6252,6 +6576,7 @@
         <v>53.17</v>
       </c>
       <c r="F275" s="7" t="inlineStr"/>
+      <c r="G275" s="7" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
@@ -6272,6 +6597,7 @@
         <v>87.43000000000001</v>
       </c>
       <c r="F276" s="7" t="inlineStr"/>
+      <c r="G276" s="7" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
@@ -6292,6 +6618,7 @@
         <v>86.76000000000001</v>
       </c>
       <c r="F277" s="7" t="inlineStr"/>
+      <c r="G277" s="7" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
@@ -6312,6 +6639,11 @@
         <v>85.23</v>
       </c>
       <c r="F278" s="7" t="inlineStr"/>
+      <c r="G278" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
@@ -6332,6 +6664,11 @@
         <v>74.11</v>
       </c>
       <c r="F279" s="7" t="inlineStr"/>
+      <c r="G279" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
@@ -6352,6 +6689,11 @@
         <v>59.17</v>
       </c>
       <c r="F280" s="7" t="inlineStr"/>
+      <c r="G280" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>